<commit_message>
Now generate Ratios at KYC level if kyc_level_data_gen is enabled in … (#1470)
* Now generate Ratios at KYC level if kyc_level_data_gen is enabled in fund

* Fixed fmv_on_date

* Fix api moic computation

* check yc before using it

* Now sum last account entry for each commitment

* Updated excel for spec to pass

* Review changes - check kyc level doc gen in jobs, override delegated methods in InvestorKycCalcs

* Update comment
</commit_message>
<xml_diff>
--- a/public/sample_uploads/fund_ratios/fund_ratios.xlsx
+++ b/public/sample_uploads/fund_ratios/fund_ratios.xlsx
@@ -124,10 +124,10 @@
     <t xml:space="preserve">TSTF2 Port Co 4  CCPS</t>
   </si>
   <si>
-    <t xml:space="preserve">210000000.0 x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">560000000.0 x</t>
+    <t xml:space="preserve">1.5 x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.0 x</t>
   </si>
   <si>
     <t xml:space="preserve">1.50 x</t>
@@ -839,7 +839,7 @@
         <v>15</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>210000000</v>
+        <v>1.5</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>34</v>
@@ -868,7 +868,7 @@
         <v>15</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>560000000</v>
+        <v>2</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>35</v>

</xml_diff>